<commit_message>
completeness: v2 opening rule, checker judges opening only
</commit_message>
<xml_diff>
--- a/eval/RBI_NBFC_Retrieval_Questions_results_v1.xlsx
+++ b/eval/RBI_NBFC_Retrieval_Questions_results_v1.xlsx
@@ -2683,12 +2683,12 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>declined to answer an in-scope question - retrieval likely missed</t>
+          <t>no numeric facts to compare - read the answer yourself</t>
         </is>
       </c>
       <c r="J42" t="n">

</xml_diff>